<commit_message>
#23 R3 and J1 Updated in BOM
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.2/BOM/ClientBOM-IoT-Button.xlsx
+++ b/Design Files/IoT-Button-v1.2/BOM/ClientBOM-IoT-Button.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="161">
   <si>
     <t>Component list</t>
   </si>
@@ -391,12 +391,6 @@
     <t>DC Power Jack</t>
   </si>
   <si>
-    <t>Panel Mounting DC Power Receptacle 260℃ Brass -20℃~+70℃ 2mm 6mm 2.5A 24V SMD AC/DC Power Connectors ROHS</t>
-  </si>
-  <si>
-    <t>DC-044D-2.5A-2.0-SMT</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -487,7 +481,28 @@
     <t>C1, C2, C5, C8, C10, C11, C12, C14, C15, C16, C17, C18, C20, C25, C26</t>
   </si>
   <si>
-    <t>R3, R5, R12</t>
+    <t>DC Power Receptacle 260℃ Brass -20℃~+70℃ 2.5mm 6mm 2.5A 24V Plugin AC/DC Power Connectors ROHS</t>
+  </si>
+  <si>
+    <t>DC-0360-2.5</t>
+  </si>
+  <si>
+    <t>R5, R12</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>RES 56K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-0756KL</t>
+  </si>
+  <si>
+    <t>56k</t>
   </si>
 </sst>
 </file>
@@ -1474,7 +1489,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="22" customWidth="1"/>
@@ -1485,7 +1500,7 @@
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.42578125" customWidth="1"/>
   </cols>
@@ -1664,7 +1679,7 @@
         <v>7</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E10" s="51" t="s">
         <v>112</v>
@@ -1685,15 +1700,15 @@
         <v>15</v>
       </c>
       <c r="K10" s="51">
-        <f t="shared" ref="K10:K11" si="0">J10*5</f>
-        <v>75</v>
+        <f>J10*2</f>
+        <v>30</v>
       </c>
       <c r="L10" s="28"/>
     </row>
     <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="49">
-        <f t="shared" ref="B11:B35" si="1">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B36" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="40" t="s">
@@ -1721,8 +1736,8 @@
         <v>6</v>
       </c>
       <c r="K11" s="51">
-        <f t="shared" si="0"/>
-        <v>30</v>
+        <f>J11*2</f>
+        <v>12</v>
       </c>
       <c r="L11" s="28"/>
     </row>
@@ -1756,9 +1771,9 @@
       <c r="J12" s="27">
         <v>2</v>
       </c>
-      <c r="K12" s="50">
-        <f>J12*5</f>
-        <v>10</v>
+      <c r="K12" s="51">
+        <f t="shared" ref="K12:K39" si="1">J12*2</f>
+        <v>4</v>
       </c>
       <c r="L12" s="27"/>
     </row>
@@ -1792,16 +1807,16 @@
       <c r="J13" s="27">
         <v>1</v>
       </c>
-      <c r="K13" s="50">
-        <f>J13*5</f>
-        <v>5</v>
+      <c r="K13" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L13" s="27"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C14" s="40" t="s">
@@ -1829,8 +1844,8 @@
         <v>1</v>
       </c>
       <c r="K14" s="51">
-        <f t="shared" ref="K14" si="2">J14*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L14" s="28"/>
     </row>
@@ -1864,16 +1879,16 @@
       <c r="J15" s="27">
         <v>1</v>
       </c>
-      <c r="K15" s="50">
-        <f>J15*5</f>
-        <v>5</v>
+      <c r="K15" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L15" s="27"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="40" t="s">
@@ -1901,8 +1916,8 @@
         <v>1</v>
       </c>
       <c r="K16" s="51">
-        <f t="shared" ref="K16" si="3">J16*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L16" s="28"/>
     </row>
@@ -1915,17 +1930,17 @@
       <c r="C17" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="50" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="G17" s="50" t="s">
-        <v>124</v>
+      <c r="E17" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>154</v>
       </c>
       <c r="H17" s="27" t="s">
         <v>88</v>
@@ -1936,23 +1951,23 @@
       <c r="J17" s="27">
         <v>1</v>
       </c>
-      <c r="K17" s="50">
-        <f>J17*5</f>
-        <v>5</v>
+      <c r="K17" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L17" s="27"/>
     </row>
     <row r="18" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E18" s="51" t="s">
         <v>39</v>
@@ -1973,8 +1988,8 @@
         <v>1</v>
       </c>
       <c r="K18" s="51">
-        <f t="shared" ref="K18" si="4">J18*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L18" s="28"/>
     </row>
@@ -1994,7 +2009,7 @@
         <v>40</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G19" s="50" t="s">
         <v>69</v>
@@ -2008,16 +2023,16 @@
       <c r="J19" s="27">
         <v>1</v>
       </c>
-      <c r="K19" s="50">
-        <f>J19*5</f>
-        <v>5</v>
+      <c r="K19" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L19" s="27"/>
     </row>
     <row r="20" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="40" t="s">
@@ -2045,8 +2060,8 @@
         <v>1</v>
       </c>
       <c r="K20" s="51">
-        <f t="shared" ref="K20" si="5">J20*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L20" s="28"/>
     </row>
@@ -2080,16 +2095,16 @@
       <c r="J21" s="27">
         <v>1</v>
       </c>
-      <c r="K21" s="50">
-        <f>J21*5</f>
-        <v>5</v>
+      <c r="K21" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L21" s="27"/>
     </row>
     <row r="22" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="40" t="s">
@@ -2117,8 +2132,8 @@
         <v>1</v>
       </c>
       <c r="K22" s="51">
-        <f t="shared" ref="K22" si="6">J22*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L22" s="28"/>
     </row>
@@ -2129,22 +2144,22 @@
         <v>14</v>
       </c>
       <c r="C23" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>125</v>
+      </c>
+      <c r="E23" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="F23" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="G23" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="H23" s="27" t="s">
         <v>128</v>
-      </c>
-      <c r="F23" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="G23" s="50" t="s">
-        <v>129</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>130</v>
       </c>
       <c r="I23" s="27" t="s">
         <v>100</v>
@@ -2152,35 +2167,35 @@
       <c r="J23" s="27">
         <v>6</v>
       </c>
-      <c r="K23" s="50">
-        <f>J23*5</f>
-        <v>30</v>
+      <c r="K23" s="51">
+        <f t="shared" si="1"/>
+        <v>12</v>
       </c>
       <c r="L23" s="27"/>
     </row>
     <row r="24" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C24" s="40" t="s">
         <v>14</v>
       </c>
       <c r="D24" s="42" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F24" s="28" t="s">
         <v>58</v>
       </c>
       <c r="G24" s="51" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H24" s="28" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I24" s="27" t="s">
         <v>100</v>
@@ -2189,8 +2204,8 @@
         <v>1</v>
       </c>
       <c r="K24" s="51">
-        <f t="shared" ref="K24" si="7">J24*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L24" s="28"/>
     </row>
@@ -2204,7 +2219,7 @@
         <v>15</v>
       </c>
       <c r="D25" s="43" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E25" s="50" t="s">
         <v>46</v>
@@ -2224,16 +2239,16 @@
       <c r="J25" s="27">
         <v>5</v>
       </c>
-      <c r="K25" s="50">
-        <f>J25*5</f>
-        <v>25</v>
+      <c r="K25" s="51">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="L25" s="27"/>
     </row>
     <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="40" t="s">
@@ -2261,470 +2276,506 @@
         <v>1</v>
       </c>
       <c r="K26" s="51">
-        <f t="shared" ref="K26" si="8">J26*5</f>
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L26" s="28"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="49">
-        <f>ROW(B27) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C27" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="43" t="s">
-        <v>155</v>
-      </c>
-      <c r="E27" s="50" t="s">
-        <v>135</v>
-      </c>
-      <c r="F27" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G27" s="50" t="s">
-        <v>136</v>
-      </c>
-      <c r="H27" s="27" t="s">
+      <c r="D27" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="E27" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="F27" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>159</v>
+      </c>
+      <c r="H27" s="28" t="s">
         <v>80</v>
       </c>
       <c r="I27" s="50" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="J27" s="27">
-        <v>3</v>
-      </c>
-      <c r="K27" s="50">
-        <f>J27*5</f>
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="K27" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L27" s="27"/>
     </row>
     <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D28" s="42" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="F28" s="28" t="s">
+      <c r="D28" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G28" s="51" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" s="28" t="s">
+      <c r="G28" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="H28" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="I28" s="51" t="s">
-        <v>96</v>
-      </c>
-      <c r="J28" s="28">
-        <v>1</v>
+      <c r="I28" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="J28" s="27">
+        <v>2</v>
       </c>
       <c r="K28" s="51">
-        <f t="shared" ref="K28" si="9">J28*5</f>
-        <v>5</v>
-      </c>
-      <c r="L28" s="28"/>
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="L28" s="27"/>
     </row>
     <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="49">
-        <f>ROW(B29) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="E29" s="50" t="s">
-        <v>47</v>
-      </c>
-      <c r="F29" s="27" t="s">
+      <c r="D29" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="G29" s="50" t="s">
-        <v>76</v>
-      </c>
-      <c r="H29" s="27" t="s">
+      <c r="G29" s="51" t="s">
+        <v>74</v>
+      </c>
+      <c r="H29" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="I29" s="50" t="s">
-        <v>98</v>
-      </c>
-      <c r="J29" s="27">
-        <v>1</v>
-      </c>
-      <c r="K29" s="50">
-        <f>J29*5</f>
-        <v>5</v>
-      </c>
-      <c r="L29" s="27"/>
+      <c r="I29" s="51" t="s">
+        <v>96</v>
+      </c>
+      <c r="J29" s="28">
+        <v>1</v>
+      </c>
+      <c r="K29" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L29" s="28"/>
     </row>
     <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D30" s="42" t="s">
-        <v>138</v>
-      </c>
-      <c r="E30" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="F30" s="28" t="s">
+      <c r="D30" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="F30" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G30" s="51" t="s">
-        <v>75</v>
-      </c>
-      <c r="H30" s="28" t="s">
+      <c r="G30" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H30" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="I30" s="51" t="s">
-        <v>151</v>
-      </c>
-      <c r="J30" s="28">
+      <c r="I30" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="J30" s="27">
         <v>1</v>
       </c>
       <c r="K30" s="51">
-        <f t="shared" ref="K30:K31" si="10">J30*5</f>
-        <v>5</v>
-      </c>
-      <c r="L30" s="28"/>
-    </row>
-    <row r="31" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L30" s="27"/>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="49">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="E31" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="G31" s="51" t="s">
+        <v>75</v>
+      </c>
+      <c r="H31" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I31" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="J31" s="28">
+        <v>1</v>
+      </c>
+      <c r="K31" s="51">
         <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-      <c r="C31" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="D31" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="51" t="s">
-        <v>141</v>
-      </c>
-      <c r="F31" s="28" t="s">
-        <v>142</v>
-      </c>
-      <c r="G31" s="51" t="s">
-        <v>142</v>
-      </c>
-      <c r="H31" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="I31" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J31" s="28">
-        <v>1</v>
-      </c>
-      <c r="K31" s="51">
-        <f t="shared" si="10"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L31" s="28"/>
     </row>
-    <row r="32" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="49">
-        <f>ROW(B32) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="F32" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="43" t="s">
-        <v>143</v>
-      </c>
-      <c r="E32" s="50" t="s">
-        <v>144</v>
-      </c>
-      <c r="F32" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="G32" s="50" t="s">
-        <v>145</v>
-      </c>
-      <c r="H32" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="J32" s="27">
+      <c r="G32" s="51" t="s">
+        <v>140</v>
+      </c>
+      <c r="H32" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="I32" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J32" s="28">
+        <v>1</v>
+      </c>
+      <c r="K32" s="51">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="K32" s="50">
-        <f>J32*5</f>
-        <v>10</v>
-      </c>
-      <c r="L32" s="27"/>
+      <c r="L32" s="28"/>
     </row>
     <row r="33" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="49">
+        <f>ROW(B33) - ROW($B$9)</f>
+        <v>24</v>
+      </c>
+      <c r="C33" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="H33" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="I33" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="J33" s="27">
+        <v>2</v>
+      </c>
+      <c r="K33" s="51">
         <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-      <c r="C33" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="D33" s="42" t="s">
-        <v>147</v>
-      </c>
-      <c r="E33" s="51" t="s">
-        <v>148</v>
-      </c>
-      <c r="F33" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="G33" s="51" t="s">
-        <v>149</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="I33" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J33" s="28">
-        <v>1</v>
-      </c>
-      <c r="K33" s="51">
-        <f t="shared" ref="K33" si="11">J33*5</f>
-        <v>5</v>
-      </c>
-      <c r="L33" s="28"/>
-    </row>
-    <row r="34" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="L33" s="27"/>
+    </row>
+    <row r="34" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="49">
-        <f>ROW(B34) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="G34" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="H34" s="27" t="s">
-        <v>89</v>
+        <v>138</v>
+      </c>
+      <c r="D34" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E34" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="F34" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="G34" s="51" t="s">
+        <v>147</v>
+      </c>
+      <c r="H34" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="I34" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="J34" s="27">
-        <v>1</v>
-      </c>
-      <c r="K34" s="50">
-        <f>J34*5</f>
-        <v>5</v>
-      </c>
-      <c r="L34" s="27"/>
-    </row>
-    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J34" s="28">
+        <v>1</v>
+      </c>
+      <c r="K34" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L34" s="28"/>
+    </row>
+    <row r="35" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="49">
+        <f>ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="G35" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="I35" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J35" s="27">
+        <v>1</v>
+      </c>
+      <c r="K35" s="51">
         <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-      <c r="C35" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="42" t="s">
-        <v>31</v>
-      </c>
-      <c r="E35" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="F35" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="G35" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="H35" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="I35" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J35" s="28">
-        <v>1</v>
-      </c>
-      <c r="K35" s="51">
-        <f t="shared" ref="K35" si="12">J35*5</f>
-        <v>5</v>
-      </c>
-      <c r="L35" s="28"/>
-    </row>
-    <row r="36" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="L35" s="27"/>
+    </row>
+    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="49">
-        <f>ROW(B36) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C36" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="F36" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="G36" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="H36" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I36" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J36" s="28">
+        <v>1</v>
+      </c>
+      <c r="K36" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L36" s="28"/>
+    </row>
+    <row r="37" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="49">
+        <f>ROW(B37) - ROW($B$9)</f>
+        <v>28</v>
+      </c>
+      <c r="C37" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="43" t="s">
+      <c r="D37" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="50" t="s">
+      <c r="E37" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F37" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="G36" s="50" t="s">
+      <c r="G37" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="H36" s="27" t="s">
+      <c r="H37" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="I36" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J36" s="27">
-        <v>1</v>
-      </c>
-      <c r="K36" s="50">
-        <f>J36*5</f>
-        <v>5</v>
-      </c>
-      <c r="L36" s="27"/>
-    </row>
-    <row r="37" spans="1:12" ht="48" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="B37" s="39">
-        <f t="shared" ref="B37:B38" si="13">ROW(B37) - ROW($B$9)</f>
-        <v>28</v>
-      </c>
-      <c r="C37" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="D37" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="F37" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="G37" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="H37" s="27" t="s">
-        <v>100</v>
-      </c>
       <c r="I37" s="27" t="s">
         <v>100</v>
       </c>
       <c r="J37" s="27">
         <v>1</v>
       </c>
-      <c r="K37" s="27">
-        <f>J37*5</f>
-        <v>5</v>
+      <c r="K37" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
       <c r="L37" s="27"/>
     </row>
-    <row r="38" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" ht="48" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="39">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="B38:B39" si="2">ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="40" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D38" s="27" t="s">
         <v>107</v>
       </c>
       <c r="E38" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G38" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H38" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="I38" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J38" s="27">
+        <v>1</v>
+      </c>
+      <c r="K38" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L38" s="27"/>
+    </row>
+    <row r="39" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1"/>
+      <c r="B39" s="39">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="C39" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E39" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="F38" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="G38" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="H38" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="I38" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J38" s="27">
-        <v>1</v>
-      </c>
-      <c r="K38" s="27">
-        <f>J38*5</f>
-        <v>5</v>
-      </c>
-      <c r="L38" s="28"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-      <c r="B39" s="52"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="57"/>
-      <c r="J39" s="57"/>
-      <c r="K39" s="57"/>
-      <c r="L39" s="58"/>
-    </row>
-    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="I39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J39" s="27">
+        <v>1</v>
+      </c>
+      <c r="K39" s="51">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L39" s="28"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="44"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
-      <c r="J40" s="47"/>
-      <c r="K40" s="47"/>
-      <c r="L40" s="59"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="53"/>
+      <c r="D40" s="54"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="57"/>
+      <c r="J40" s="57"/>
+      <c r="K40" s="57"/>
+      <c r="L40" s="58"/>
+    </row>
+    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
+      <c r="B41" s="44"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="47"/>
+      <c r="F41" s="47"/>
+      <c r="G41" s="47"/>
+      <c r="H41" s="47"/>
+      <c r="I41" s="47"/>
+      <c r="J41" s="47"/>
+      <c r="K41" s="47"/>
+      <c r="L41" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2739,7 +2790,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -2929,7 +2980,7 @@
         <v>7</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E10" s="51" t="s">
         <v>112</v>
@@ -2958,7 +3009,7 @@
     <row r="11" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="49">
-        <f t="shared" ref="B11:B35" si="1">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B36" si="1">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="40" t="s">
@@ -3171,7 +3222,7 @@
       </c>
       <c r="L16" s="28"/>
     </row>
-    <row r="17" spans="1:12" s="41" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="49">
         <f>ROW(B17) - ROW($B$9)</f>
@@ -3180,17 +3231,17 @@
       <c r="C17" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="50" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="G17" s="50" t="s">
-        <v>124</v>
+      <c r="E17" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>154</v>
       </c>
       <c r="H17" s="27" t="s">
         <v>88</v>
@@ -3217,7 +3268,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E18" s="51" t="s">
         <v>39</v>
@@ -3259,7 +3310,7 @@
         <v>40</v>
       </c>
       <c r="F19" s="27" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G19" s="50" t="s">
         <v>69</v>
@@ -3394,22 +3445,22 @@
         <v>14</v>
       </c>
       <c r="C23" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>125</v>
+      </c>
+      <c r="E23" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="F23" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="G23" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="H23" s="27" t="s">
         <v>128</v>
-      </c>
-      <c r="F23" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="G23" s="50" t="s">
-        <v>129</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>130</v>
       </c>
       <c r="I23" s="27" t="s">
         <v>100</v>
@@ -3433,19 +3484,19 @@
         <v>14</v>
       </c>
       <c r="D24" s="42" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F24" s="28" t="s">
         <v>58</v>
       </c>
       <c r="G24" s="51" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H24" s="28" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I24" s="27" t="s">
         <v>100</v>
@@ -3469,7 +3520,7 @@
         <v>15</v>
       </c>
       <c r="D25" s="43" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E25" s="50" t="s">
         <v>46</v>
@@ -3526,7 +3577,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="51">
-        <f t="shared" ref="K26" si="9">J26*5</f>
+        <f t="shared" ref="K26:K27" si="9">J26*5</f>
         <v>5</v>
       </c>
       <c r="L26" s="28"/>
@@ -3534,413 +3585,413 @@
     <row r="27" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="49">
-        <f>ROW(B27) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C27" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="43" t="s">
-        <v>155</v>
-      </c>
-      <c r="E27" s="50" t="s">
-        <v>135</v>
-      </c>
-      <c r="F27" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G27" s="50" t="s">
-        <v>136</v>
-      </c>
-      <c r="H27" s="27" t="s">
+      <c r="D27" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="E27" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="F27" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>159</v>
+      </c>
+      <c r="H27" s="28" t="s">
         <v>80</v>
       </c>
       <c r="I27" s="50" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="J27" s="27">
-        <v>3</v>
-      </c>
-      <c r="K27" s="50">
-        <f>J27*5</f>
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="K27" s="51">
+        <f t="shared" si="9"/>
+        <v>5</v>
       </c>
       <c r="L27" s="27"/>
     </row>
     <row r="28" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D28" s="42" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="F28" s="28" t="s">
+      <c r="D28" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="E28" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G28" s="51" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" s="28" t="s">
+      <c r="G28" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="H28" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="I28" s="51" t="s">
-        <v>96</v>
-      </c>
-      <c r="J28" s="28">
-        <v>1</v>
-      </c>
-      <c r="K28" s="51">
-        <f t="shared" ref="K28" si="10">J28*5</f>
-        <v>5</v>
-      </c>
-      <c r="L28" s="28"/>
+      <c r="I28" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="J28" s="27">
+        <v>2</v>
+      </c>
+      <c r="K28" s="50">
+        <f>J28*5</f>
+        <v>10</v>
+      </c>
+      <c r="L28" s="27"/>
     </row>
     <row r="29" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="49">
-        <f>ROW(B29) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="E29" s="50" t="s">
-        <v>47</v>
-      </c>
-      <c r="F29" s="27" t="s">
+      <c r="D29" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="G29" s="50" t="s">
-        <v>76</v>
-      </c>
-      <c r="H29" s="27" t="s">
+      <c r="G29" s="51" t="s">
+        <v>74</v>
+      </c>
+      <c r="H29" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="I29" s="50" t="s">
-        <v>98</v>
-      </c>
-      <c r="J29" s="27">
-        <v>1</v>
-      </c>
-      <c r="K29" s="50">
-        <f>J29*5</f>
+      <c r="I29" s="51" t="s">
+        <v>96</v>
+      </c>
+      <c r="J29" s="28">
+        <v>1</v>
+      </c>
+      <c r="K29" s="51">
+        <f t="shared" ref="K29" si="10">J29*5</f>
         <v>5</v>
       </c>
-      <c r="L29" s="27"/>
+      <c r="L29" s="28"/>
     </row>
     <row r="30" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="D30" s="42" t="s">
-        <v>138</v>
-      </c>
-      <c r="E30" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="F30" s="28" t="s">
+      <c r="D30" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="F30" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G30" s="51" t="s">
-        <v>75</v>
-      </c>
-      <c r="H30" s="28" t="s">
+      <c r="G30" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="H30" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="I30" s="51" t="s">
-        <v>151</v>
-      </c>
-      <c r="J30" s="28">
-        <v>1</v>
-      </c>
-      <c r="K30" s="51">
-        <f t="shared" ref="K30" si="11">J30*5</f>
+      <c r="I30" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="J30" s="27">
+        <v>1</v>
+      </c>
+      <c r="K30" s="50">
+        <f>J30*5</f>
         <v>5</v>
       </c>
-      <c r="L30" s="28"/>
-    </row>
-    <row r="31" spans="1:12" s="41" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L30" s="27"/>
+    </row>
+    <row r="31" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="49">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C31" s="40" t="s">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="D31" s="42" t="s">
-        <v>29</v>
+        <v>136</v>
       </c>
       <c r="E31" s="51" t="s">
-        <v>141</v>
+        <v>46</v>
       </c>
       <c r="F31" s="28" t="s">
-        <v>142</v>
+        <v>59</v>
       </c>
       <c r="G31" s="51" t="s">
-        <v>142</v>
+        <v>75</v>
       </c>
       <c r="H31" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="I31" s="27" t="s">
-        <v>100</v>
+        <v>80</v>
+      </c>
+      <c r="I31" s="51" t="s">
+        <v>149</v>
       </c>
       <c r="J31" s="28">
         <v>1</v>
       </c>
       <c r="K31" s="51">
-        <f t="shared" ref="K31" si="12">J31*5</f>
+        <f t="shared" ref="K31" si="11">J31*5</f>
         <v>5</v>
       </c>
       <c r="L31" s="28"/>
     </row>
-    <row r="32" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" s="41" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="49">
-        <f>ROW(B32) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="C32" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="F32" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="43" t="s">
-        <v>143</v>
-      </c>
-      <c r="E32" s="50" t="s">
-        <v>144</v>
-      </c>
-      <c r="F32" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="G32" s="50" t="s">
-        <v>145</v>
-      </c>
-      <c r="H32" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="J32" s="27">
-        <v>2</v>
-      </c>
-      <c r="K32" s="50">
-        <f>J32*5</f>
-        <v>10</v>
-      </c>
-      <c r="L32" s="27"/>
+      <c r="G32" s="51" t="s">
+        <v>140</v>
+      </c>
+      <c r="H32" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="I32" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J32" s="28">
+        <v>1</v>
+      </c>
+      <c r="K32" s="51">
+        <f t="shared" ref="K32" si="12">J32*5</f>
+        <v>5</v>
+      </c>
+      <c r="L32" s="28"/>
     </row>
     <row r="33" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
       <c r="C33" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="D33" s="42" t="s">
-        <v>147</v>
-      </c>
-      <c r="E33" s="51" t="s">
-        <v>148</v>
-      </c>
-      <c r="F33" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="G33" s="51" t="s">
-        <v>149</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="I33" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J33" s="28">
-        <v>1</v>
-      </c>
-      <c r="K33" s="51">
-        <f t="shared" ref="K33" si="13">J33*5</f>
-        <v>5</v>
-      </c>
-      <c r="L33" s="28"/>
-    </row>
-    <row r="34" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+      <c r="D33" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="E33" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="H33" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="I33" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="J33" s="27">
+        <v>2</v>
+      </c>
+      <c r="K33" s="50">
+        <f>J33*5</f>
+        <v>10</v>
+      </c>
+      <c r="L33" s="27"/>
+    </row>
+    <row r="34" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="49">
-        <f>ROW(B34) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="C34" s="40" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="G34" s="50" t="s">
-        <v>77</v>
-      </c>
-      <c r="H34" s="27" t="s">
-        <v>89</v>
+        <v>138</v>
+      </c>
+      <c r="D34" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E34" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="F34" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="G34" s="51" t="s">
+        <v>147</v>
+      </c>
+      <c r="H34" s="28" t="s">
+        <v>87</v>
       </c>
       <c r="I34" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="J34" s="27">
-        <v>1</v>
-      </c>
-      <c r="K34" s="50">
-        <f>J34*5</f>
+      <c r="J34" s="28">
+        <v>1</v>
+      </c>
+      <c r="K34" s="51">
+        <f t="shared" ref="K34" si="13">J34*5</f>
         <v>5</v>
       </c>
-      <c r="L34" s="27"/>
-    </row>
-    <row r="35" spans="1:12" s="41" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L34" s="28"/>
+    </row>
+    <row r="35" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="49">
-        <f t="shared" si="1"/>
+        <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="42" t="s">
-        <v>31</v>
-      </c>
-      <c r="E35" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="F35" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="G35" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="H35" s="28" t="s">
-        <v>90</v>
+        <v>14</v>
+      </c>
+      <c r="D35" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="G35" s="50" t="s">
+        <v>77</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>89</v>
       </c>
       <c r="I35" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="J35" s="28">
-        <v>1</v>
-      </c>
-      <c r="K35" s="51">
-        <f t="shared" ref="K35" si="14">J35*5</f>
+      <c r="J35" s="27">
+        <v>1</v>
+      </c>
+      <c r="K35" s="50">
+        <f>J35*5</f>
         <v>5</v>
       </c>
-      <c r="L35" s="28"/>
-    </row>
-    <row r="36" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L35" s="27"/>
+    </row>
+    <row r="36" spans="1:12" s="41" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="49">
-        <f>ROW(B36) - ROW($B$9)</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="C36" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="F36" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="G36" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="H36" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I36" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J36" s="28">
+        <v>1</v>
+      </c>
+      <c r="K36" s="51">
+        <f t="shared" ref="K36" si="14">J36*5</f>
+        <v>5</v>
+      </c>
+      <c r="L36" s="28"/>
+    </row>
+    <row r="37" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="49">
+        <f>ROW(B37) - ROW($B$9)</f>
+        <v>28</v>
+      </c>
+      <c r="C37" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="43" t="s">
+      <c r="D37" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="50" t="s">
+      <c r="E37" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F37" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="G36" s="50" t="s">
+      <c r="G37" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="H36" s="27" t="s">
+      <c r="H37" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="I36" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="J36" s="27">
-        <v>1</v>
-      </c>
-      <c r="K36" s="50">
-        <f>J36*5</f>
-        <v>5</v>
-      </c>
-      <c r="L36" s="27"/>
-    </row>
-    <row r="37" spans="1:12" s="41" customFormat="1" ht="48" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="B37" s="39">
-        <f t="shared" ref="B37:B38" si="15">ROW(B37) - ROW($B$9)</f>
-        <v>28</v>
-      </c>
-      <c r="C37" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="D37" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="27" t="s">
-        <v>109</v>
-      </c>
-      <c r="F37" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="G37" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="H37" s="27" t="s">
-        <v>100</v>
-      </c>
       <c r="I37" s="27" t="s">
         <v>100</v>
       </c>
       <c r="J37" s="27">
         <v>1</v>
       </c>
-      <c r="K37" s="27">
+      <c r="K37" s="50">
         <f>J37*5</f>
         <v>5</v>
       </c>
       <c r="L37" s="27"/>
     </row>
-    <row r="38" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" s="41" customFormat="1" ht="48" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="39">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="B38:B39" si="15">ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="40" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D38" s="27" t="s">
         <v>107</v>
       </c>
       <c r="E38" s="27" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F38" s="27" t="s">
         <v>100</v>
@@ -3961,49 +4012,71 @@
         <f>J38*5</f>
         <v>5</v>
       </c>
-      <c r="L38" s="28"/>
-    </row>
-    <row r="39" spans="1:12" s="41" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L38" s="27"/>
+    </row>
+    <row r="39" spans="1:12" s="41" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="52"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="55"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="57"/>
-      <c r="J39" s="57"/>
-      <c r="K39" s="57"/>
-      <c r="L39" s="58"/>
-    </row>
-    <row r="40" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="39">
+        <f t="shared" si="15"/>
+        <v>30</v>
+      </c>
+      <c r="C39" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="I39" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J39" s="27">
+        <v>1</v>
+      </c>
+      <c r="K39" s="27">
+        <f>J39*5</f>
+        <v>5</v>
+      </c>
+      <c r="L39" s="28"/>
+    </row>
+    <row r="40" spans="1:12" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="44"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
-      <c r="J40" s="47"/>
-      <c r="K40" s="47"/>
-      <c r="L40" s="59"/>
-    </row>
-    <row r="41" spans="1:12" s="41" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
-      <c r="I41"/>
-      <c r="J41"/>
-      <c r="K41"/>
-      <c r="L41"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="53"/>
+      <c r="D40" s="54"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="57"/>
+      <c r="J40" s="57"/>
+      <c r="K40" s="57"/>
+      <c r="L40" s="58"/>
+    </row>
+    <row r="41" spans="1:12" s="41" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
+      <c r="B41" s="44"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="47"/>
+      <c r="F41" s="47"/>
+      <c r="G41" s="47"/>
+      <c r="H41" s="47"/>
+      <c r="I41" s="47"/>
+      <c r="J41" s="47"/>
+      <c r="K41" s="47"/>
+      <c r="L41" s="59"/>
     </row>
     <row r="42" spans="1:12" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42"/>
@@ -4033,12 +4106,27 @@
       <c r="K43"/>
       <c r="L43"/>
     </row>
+    <row r="44" spans="1:12" s="41" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44"/>
+      <c r="B44"/>
+      <c r="C44"/>
+      <c r="D44"/>
+      <c r="E44"/>
+      <c r="F44"/>
+      <c r="G44"/>
+      <c r="H44"/>
+      <c r="I44"/>
+      <c r="J44"/>
+      <c r="K44"/>
+      <c r="L44"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="L3:L8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>